<commit_message>
Cleaned the backend code
</commit_message>
<xml_diff>
--- a/backend/exports/fouad_farm_report_2026-09.xlsx
+++ b/backend/exports/fouad_farm_report_2026-09.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:D5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -457,34 +457,66 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>كلية</t>
+          <t>شتة برتقال</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>300</v>
+        <v>1</v>
       </c>
       <c r="D2" t="n">
-        <v>74675</v>
+        <v>89</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>كلية</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>300</v>
+      </c>
+      <c r="D3" t="n">
+        <v>74675</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>كليةo</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>5120</v>
+      </c>
+      <c r="D4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
         <v>1</v>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B5" t="inlineStr">
         <is>
           <t>شتلة برتقال</t>
         </is>
       </c>
-      <c r="C3" t="n">
+      <c r="C5" t="n">
         <v>2.5</v>
       </c>
-      <c r="D3" t="n">
-        <v>33102</v>
+      <c r="D5" t="n">
+        <v>33100</v>
       </c>
     </row>
   </sheetData>
@@ -498,7 +530,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I5"/>
+  <dimension ref="A1:I6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -561,11 +593,11 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>شتلة برتقال</t>
+          <t>كلية</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -575,7 +607,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -584,50 +616,50 @@
         </is>
       </c>
       <c r="F2" t="n">
-        <v>52103</v>
+        <v>200</v>
       </c>
       <c r="G2" t="n">
-        <v>20000</v>
+        <v>0</v>
       </c>
       <c r="H2" t="n">
-        <v>32103</v>
+        <v>200</v>
       </c>
       <c r="I2" s="2" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>شتلة برتقال</t>
+          <t>كلية</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>747</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>474</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>4\4\</t>
         </is>
       </c>
       <c r="F3" t="n">
-        <v>999</v>
+        <v>74475</v>
       </c>
       <c r="G3" t="n">
         <v>0</v>
       </c>
       <c r="H3" t="n">
-        <v>999</v>
+        <v>74475</v>
       </c>
       <c r="I3" s="2" t="n">
         <v>46281</v>
@@ -635,48 +667,48 @@
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>كلية</t>
+          <t>شتة برتقال</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>747</t>
+          <t>1</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>474</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>4\4\</t>
+          <t>3</t>
         </is>
       </c>
       <c r="F4" t="n">
-        <v>74475</v>
+        <v>89</v>
       </c>
       <c r="G4" t="n">
         <v>0</v>
       </c>
       <c r="H4" t="n">
-        <v>74475</v>
+        <v>89</v>
       </c>
       <c r="I4" s="2" t="n">
-        <v>46281</v>
+        <v>46289</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>كلية</t>
+          <t>شتلة برتقال</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -686,25 +718,62 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="F5" t="n">
+        <v>52103</v>
+      </c>
+      <c r="G5" t="n">
+        <v>20000</v>
+      </c>
+      <c r="H5" t="n">
+        <v>32103</v>
+      </c>
+      <c r="I5" s="2" t="n">
+        <v>46281</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>شتلة برتقال</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
           <t>5</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
+      <c r="E6" t="inlineStr">
         <is>
           <t>7</t>
         </is>
       </c>
-      <c r="F5" t="n">
-        <v>200</v>
-      </c>
-      <c r="G5" t="n">
+      <c r="F6" t="n">
+        <v>997</v>
+      </c>
+      <c r="G6" t="n">
         <v>0</v>
       </c>
-      <c r="H5" t="n">
-        <v>200</v>
-      </c>
-      <c r="I5" s="2" t="n">
-        <v>46282</v>
+      <c r="H6" t="n">
+        <v>997</v>
+      </c>
+      <c r="I6" s="2" t="n">
+        <v>46281</v>
       </c>
     </row>
   </sheetData>
@@ -718,15 +787,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H3"/>
+  <dimension ref="A1:H5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="26" customWidth="1" min="4" max="4"/>
-    <col width="9" customWidth="1" min="5" max="5"/>
-    <col width="9" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
     <col width="11" customWidth="1" min="7" max="7"/>
     <col width="12" customWidth="1" min="8" max="8"/>
   </cols>
@@ -826,12 +895,76 @@
         <v>29702.5</v>
       </c>
       <c r="F3" t="n">
-        <v>21702.5</v>
+        <v>29702.5</v>
       </c>
       <c r="G3" t="n">
-        <v>8000</v>
+        <v>0</v>
       </c>
       <c r="H3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>5</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>ll</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="n">
+        <v>46289</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>شتة برتقال x11</t>
+        </is>
+      </c>
+      <c r="E4" t="n">
+        <v>15</v>
+      </c>
+      <c r="F4" t="n">
+        <v>7</v>
+      </c>
+      <c r="G4" t="n">
+        <v>8</v>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>6</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>ll</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="n">
+        <v>46289</v>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>شتلة برتقال x2</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>5</v>
+      </c>
+      <c r="F5" t="n">
+        <v>2</v>
+      </c>
+      <c r="G5" t="n">
+        <v>3</v>
+      </c>
+      <c r="H5" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -848,13 +981,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:E8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="9" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
@@ -967,6 +1100,69 @@
       </c>
       <c r="E5" s="2" t="n">
         <v>46282</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>ll</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Deposit</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>7</v>
+      </c>
+      <c r="E6" s="2" t="n">
+        <v>46289</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>4</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>hh</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Regular</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>8000</v>
+      </c>
+      <c r="E7" s="2" t="n">
+        <v>46289</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>6</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>ll</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Deposit</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>2</v>
+      </c>
+      <c r="E8" s="2" t="n">
+        <v>46289</v>
       </c>
     </row>
   </sheetData>
@@ -980,7 +1176,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:D4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1024,22 +1220,38 @@
         <v>29702.5</v>
       </c>
       <c r="D2" t="n">
-        <v>21702.5</v>
+        <v>29702.5</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
+          <t>ll</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>2</v>
+      </c>
+      <c r="C3" t="n">
+        <v>20</v>
+      </c>
+      <c r="D3" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
           <t>خخ</t>
         </is>
       </c>
-      <c r="B3" t="n">
+      <c r="B4" t="n">
         <v>1</v>
       </c>
-      <c r="C3" t="n">
+      <c r="C4" t="n">
         <v>2.5</v>
       </c>
-      <c r="D3" t="n">
+      <c r="D4" t="n">
         <v>2.5</v>
       </c>
     </row>

</xml_diff>